<commit_message>
all order files updated upto 15 sep 2026 Tuesday
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/order_files/FullOrders_upto_11sep26_Fri.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/order_files/FullOrders_upto_11sep26_Fri.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\order_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14B6B1A-CA60-47B6-8DC2-D70C476504AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8185570C-B780-4695-B0A8-4022A1306DC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1103,7 +1103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1278,28 +1278,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="22" fontId="1" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -1725,7 +1703,7 @@
         <v>34175</v>
       </c>
       <c r="N2" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B2, $C$2:$C$767, C2, $D$2:$D$767, D2, $E$2:$E$767, E2) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N2:N65" si="0">IF(COUNTIFS( $B$2:$B$767, B2, $C$2:$C$767, C2, $D$2:$D$767, D2, $E$2:$E$767, E2) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
       <c r="O2" s="10"/>
@@ -1766,7 +1744,7 @@
       <c r="L3" s="17"/>
       <c r="M3" s="17"/>
       <c r="N3" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B3, $C$2:$C$767, C3, $D$2:$D$767, D3, $E$2:$E$767, E3) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O3" s="10"/>
@@ -1807,7 +1785,7 @@
       <c r="L4" s="17"/>
       <c r="M4" s="17"/>
       <c r="N4" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B4, $C$2:$C$767, C4, $D$2:$D$767, D4, $E$2:$E$767, E4) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O4" s="10"/>
@@ -1848,7 +1826,7 @@
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
       <c r="N5" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B5, $C$2:$C$767, C5, $D$2:$D$767, D5, $E$2:$E$767, E5) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O5" s="10"/>
@@ -1889,7 +1867,7 @@
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
       <c r="N6" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B6, $C$2:$C$767, C6, $D$2:$D$767, D6, $E$2:$E$767, E6) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O6" s="10"/>
@@ -1930,7 +1908,7 @@
       <c r="L7" s="17"/>
       <c r="M7" s="17"/>
       <c r="N7" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B7, $C$2:$C$767, C7, $D$2:$D$767, D7, $E$2:$E$767, E7) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O7" s="10"/>
@@ -1969,7 +1947,7 @@
       <c r="L8" s="17"/>
       <c r="M8" s="17"/>
       <c r="N8" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B8, $C$2:$C$767, C8, $D$2:$D$767, D8, $E$2:$E$767, E8) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O8" s="26"/>
@@ -2017,7 +1995,7 @@
         <v>500</v>
       </c>
       <c r="N9" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B9, $C$2:$C$767, C9, $D$2:$D$767, D9, $E$2:$E$767, E9) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O9" s="10"/>
@@ -2058,7 +2036,7 @@
       <c r="L10" s="17"/>
       <c r="M10" s="17"/>
       <c r="N10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B10, $C$2:$C$767, C10, $D$2:$D$767, D10, $E$2:$E$767, E10) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O10"/>
@@ -2097,7 +2075,7 @@
       <c r="L11" s="17"/>
       <c r="M11" s="17"/>
       <c r="N11" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B11, $C$2:$C$767, C11, $D$2:$D$767, D11, $E$2:$E$767, E11) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O11" s="19"/>
@@ -2138,7 +2116,7 @@
       <c r="L12" s="17"/>
       <c r="M12" s="17"/>
       <c r="N12" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B12, $C$2:$C$767, C12, $D$2:$D$767, D12, $E$2:$E$767, E12) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P12" s="34"/>
@@ -2178,7 +2156,7 @@
       <c r="L13" s="17"/>
       <c r="M13" s="17"/>
       <c r="N13" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B13, $C$2:$C$767, C13, $D$2:$D$767, D13, $E$2:$E$767, E13) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O13" s="10"/>
@@ -2219,7 +2197,7 @@
       <c r="L14" s="17"/>
       <c r="M14" s="17"/>
       <c r="N14" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B14, $C$2:$C$767, C14, $D$2:$D$767, D14, $E$2:$E$767, E14) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O14" s="10"/>
@@ -2267,7 +2245,7 @@
         <v>300</v>
       </c>
       <c r="N15" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B15, $C$2:$C$767, C15, $D$2:$D$767, D15, $E$2:$E$767, E15) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O15" s="10"/>
@@ -2308,7 +2286,7 @@
       <c r="L16" s="17"/>
       <c r="M16" s="17"/>
       <c r="N16" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B16, $C$2:$C$767, C16, $D$2:$D$767, D16, $E$2:$E$767, E16) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O16" s="10"/>
@@ -2347,7 +2325,7 @@
       <c r="L17" s="17"/>
       <c r="M17" s="17"/>
       <c r="N17" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B17, $C$2:$C$767, C17, $D$2:$D$767, D17, $E$2:$E$767, E17) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O17" s="10"/>
@@ -2388,7 +2366,7 @@
       <c r="L18" s="17"/>
       <c r="M18" s="17"/>
       <c r="N18" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B18, $C$2:$C$767, C18, $D$2:$D$767, D18, $E$2:$E$767, E18) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P18" s="10"/>
@@ -2428,7 +2406,7 @@
       <c r="L19" s="17"/>
       <c r="M19" s="17"/>
       <c r="N19" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B19, $C$2:$C$767, C19, $D$2:$D$767, D19, $E$2:$E$767, E19) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O19" s="10"/>
@@ -2476,7 +2454,7 @@
         <v>300</v>
       </c>
       <c r="N20" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B20, $C$2:$C$767, C20, $D$2:$D$767, D20, $E$2:$E$767, E20) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2522,7 +2500,7 @@
         <v>525</v>
       </c>
       <c r="N21" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B21, $C$2:$C$767, C21, $D$2:$D$767, D21, $E$2:$E$767, E21) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O21" s="10"/>
@@ -2561,7 +2539,7 @@
       <c r="L22" s="17"/>
       <c r="M22" s="17"/>
       <c r="N22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B22, $C$2:$C$767, C22, $D$2:$D$767, D22, $E$2:$E$767, E22) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O22" s="10"/>
@@ -2602,7 +2580,7 @@
       <c r="L23" s="17"/>
       <c r="M23" s="17"/>
       <c r="N23" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B23, $C$2:$C$767, C23, $D$2:$D$767, D23, $E$2:$E$767, E23) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O23" s="10"/>
@@ -2649,7 +2627,7 @@
         <v>300</v>
       </c>
       <c r="N24" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B24, $C$2:$C$767, C24, $D$2:$D$767, D24, $E$2:$E$767, E24) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O24" s="10"/>
@@ -2690,7 +2668,7 @@
       <c r="L25" s="17"/>
       <c r="M25" s="17"/>
       <c r="N25" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B25, $C$2:$C$767, C25, $D$2:$D$767, D25, $E$2:$E$767, E25) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O25" s="10"/>
@@ -2731,7 +2709,7 @@
       <c r="L26" s="17"/>
       <c r="M26" s="17"/>
       <c r="N26" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B26, $C$2:$C$767, C26, $D$2:$D$767, D26, $E$2:$E$767, E26) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2770,7 +2748,7 @@
       <c r="L27" s="17"/>
       <c r="M27" s="17"/>
       <c r="N27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B27, $C$2:$C$767, C27, $D$2:$D$767, D27, $E$2:$E$767, E27) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O27" s="34"/>
@@ -2810,7 +2788,7 @@
       <c r="L28" s="17"/>
       <c r="M28" s="17"/>
       <c r="N28" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B28, $C$2:$C$767, C28, $D$2:$D$767, D28, $E$2:$E$767, E28) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O28" s="10"/>
@@ -2851,7 +2829,7 @@
       <c r="L29" s="17"/>
       <c r="M29" s="17"/>
       <c r="N29" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B29, $C$2:$C$767, C29, $D$2:$D$767, D29, $E$2:$E$767, E29) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2898,7 +2876,7 @@
         <v>650</v>
       </c>
       <c r="N30" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B30, $C$2:$C$767, C30, $D$2:$D$767, D30, $E$2:$E$767, E30) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P30" s="10"/>
@@ -2938,7 +2916,7 @@
       <c r="L31" s="17"/>
       <c r="M31" s="17"/>
       <c r="N31" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B31, $C$2:$C$767, C31, $D$2:$D$767, D31, $E$2:$E$767, E31) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2977,7 +2955,7 @@
       <c r="L32" s="17"/>
       <c r="M32" s="17"/>
       <c r="N32" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B32, $C$2:$C$767, C32, $D$2:$D$767, D32, $E$2:$E$767, E32) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3016,7 +2994,7 @@
       <c r="L33" s="17"/>
       <c r="M33" s="17"/>
       <c r="N33" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B33, $C$2:$C$767, C33, $D$2:$D$767, D33, $E$2:$E$767, E33) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3055,7 +3033,7 @@
       <c r="L34" s="17"/>
       <c r="M34" s="17"/>
       <c r="N34" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B34, $C$2:$C$767, C34, $D$2:$D$767, D34, $E$2:$E$767, E34) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3092,7 +3070,7 @@
       <c r="L35" s="17"/>
       <c r="M35" s="17"/>
       <c r="N35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B35, $C$2:$C$767, C35, $D$2:$D$767, D35, $E$2:$E$767, E35) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P35" s="10"/>
@@ -3139,7 +3117,7 @@
         <v>516</v>
       </c>
       <c r="N36" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B36, $C$2:$C$767, C36, $D$2:$D$767, D36, $E$2:$E$767, E36) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O36" s="10"/>
@@ -3187,7 +3165,7 @@
         <v>300</v>
       </c>
       <c r="N37" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B37, $C$2:$C$767, C37, $D$2:$D$767, D37, $E$2:$E$767, E37) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O37" s="10"/>
@@ -3226,7 +3204,7 @@
       <c r="L38" s="17"/>
       <c r="M38" s="17"/>
       <c r="N38" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B38, $C$2:$C$767, C38, $D$2:$D$767, D38, $E$2:$E$767, E38) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P38" s="10"/>
@@ -3266,7 +3244,7 @@
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
       <c r="N39" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B39, $C$2:$C$767, C39, $D$2:$D$767, D39, $E$2:$E$767, E39) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O39" s="10"/>
@@ -3307,7 +3285,7 @@
       <c r="L40" s="17"/>
       <c r="M40" s="17"/>
       <c r="N40" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B40, $C$2:$C$767, C40, $D$2:$D$767, D40, $E$2:$E$767, E40) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3344,7 +3322,7 @@
       <c r="L41" s="17"/>
       <c r="M41" s="17"/>
       <c r="N41" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B41, $C$2:$C$767, C41, $D$2:$D$767, D41, $E$2:$E$767, E41) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O41"/>
@@ -3392,7 +3370,7 @@
         <v>460</v>
       </c>
       <c r="N42" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B42, $C$2:$C$767, C42, $D$2:$D$767, D42, $E$2:$E$767, E42) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O42"/>
@@ -3430,7 +3408,7 @@
       <c r="L43" s="17"/>
       <c r="M43" s="17"/>
       <c r="N43" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B43, $C$2:$C$767, C43, $D$2:$D$767, D43, $E$2:$E$767, E43) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P43"/>
@@ -3470,7 +3448,7 @@
       <c r="L44" s="17"/>
       <c r="M44" s="17"/>
       <c r="N44" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B44, $C$2:$C$767, C44, $D$2:$D$767, D44, $E$2:$E$767, E44) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O44"/>
@@ -3509,7 +3487,7 @@
       <c r="L45" s="17"/>
       <c r="M45" s="17"/>
       <c r="N45" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B45, $C$2:$C$767, C45, $D$2:$D$767, D45, $E$2:$E$767, E45) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O45"/>
@@ -3557,7 +3535,7 @@
         <v>300</v>
       </c>
       <c r="N46" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B46, $C$2:$C$767, C46, $D$2:$D$767, D46, $E$2:$E$767, E46) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O46"/>
@@ -3598,7 +3576,7 @@
       <c r="L47" s="17"/>
       <c r="M47" s="17"/>
       <c r="N47" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B47, $C$2:$C$767, C47, $D$2:$D$767, D47, $E$2:$E$767, E47) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O47"/>
@@ -3639,7 +3617,7 @@
       <c r="L48" s="17"/>
       <c r="M48" s="17"/>
       <c r="N48" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B48, $C$2:$C$767, C48, $D$2:$D$767, D48, $E$2:$E$767, E48) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O48"/>
@@ -3680,7 +3658,7 @@
       <c r="L49" s="17"/>
       <c r="M49" s="17"/>
       <c r="N49" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B49, $C$2:$C$767, C49, $D$2:$D$767, D49, $E$2:$E$767, E49) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O49"/>
@@ -3721,7 +3699,7 @@
       <c r="L50" s="17"/>
       <c r="M50" s="17"/>
       <c r="N50" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B50, $C$2:$C$767, C50, $D$2:$D$767, D50, $E$2:$E$767, E50) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P50"/>
@@ -3769,7 +3747,7 @@
         <v>540</v>
       </c>
       <c r="N51" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B51, $C$2:$C$767, C51, $D$2:$D$767, D51, $E$2:$E$767, E51) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O51"/>
@@ -3808,7 +3786,7 @@
       <c r="L52" s="17"/>
       <c r="M52" s="17"/>
       <c r="N52" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B52, $C$2:$C$767, C52, $D$2:$D$767, D52, $E$2:$E$767, E52) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O52"/>
@@ -3850,7 +3828,7 @@
         <v>3156</v>
       </c>
       <c r="N53" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B53, $C$2:$C$767, C53, $D$2:$D$767, D53, $E$2:$E$767, E53) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P53" s="19"/>
@@ -3888,7 +3866,7 @@
       <c r="L54" s="17"/>
       <c r="M54" s="17"/>
       <c r="N54" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B54, $C$2:$C$767, C54, $D$2:$D$767, D54, $E$2:$E$767, E54) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O54"/>
@@ -3927,7 +3905,7 @@
       <c r="L55" s="17"/>
       <c r="M55" s="17"/>
       <c r="N55" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B55, $C$2:$C$767, C55, $D$2:$D$767, D55, $E$2:$E$767, E55) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O55"/>
@@ -3966,7 +3944,7 @@
       <c r="L56" s="17"/>
       <c r="M56" s="17"/>
       <c r="N56" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B56, $C$2:$C$767, C56, $D$2:$D$767, D56, $E$2:$E$767, E56) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O56"/>
@@ -4009,7 +3987,7 @@
       <c r="L57" s="17"/>
       <c r="M57" s="17"/>
       <c r="N57" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B57, $C$2:$C$767, C57, $D$2:$D$767, D57, $E$2:$E$767, E57) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O57"/>
@@ -4050,7 +4028,7 @@
       <c r="L58" s="17"/>
       <c r="M58" s="17"/>
       <c r="N58" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B58, $C$2:$C$767, C58, $D$2:$D$767, D58, $E$2:$E$767, E58) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O58"/>
@@ -4091,7 +4069,7 @@
       <c r="L59" s="17"/>
       <c r="M59" s="17"/>
       <c r="N59" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B59, $C$2:$C$767, C59, $D$2:$D$767, D59, $E$2:$E$767, E59) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O59"/>
@@ -4130,7 +4108,7 @@
       <c r="L60" s="17"/>
       <c r="M60" s="17"/>
       <c r="N60" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B60, $C$2:$C$767, C60, $D$2:$D$767, D60, $E$2:$E$767, E60) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O60"/>
@@ -4169,7 +4147,7 @@
       <c r="L61" s="17"/>
       <c r="M61" s="17"/>
       <c r="N61" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B61, $C$2:$C$767, C61, $D$2:$D$767, D61, $E$2:$E$767, E61) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O61"/>
@@ -4217,7 +4195,7 @@
         <v>300</v>
       </c>
       <c r="N62" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B62, $C$2:$C$767, C62, $D$2:$D$767, D62, $E$2:$E$767, E62) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O62"/>
@@ -4258,7 +4236,7 @@
       <c r="L63" s="17"/>
       <c r="M63" s="17"/>
       <c r="N63" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B63, $C$2:$C$767, C63, $D$2:$D$767, D63, $E$2:$E$767, E63) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O63"/>
@@ -4297,7 +4275,7 @@
       <c r="L64" s="17"/>
       <c r="M64" s="17"/>
       <c r="N64" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B64, $C$2:$C$767, C64, $D$2:$D$767, D64, $E$2:$E$767, E64) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O64"/>
@@ -4336,7 +4314,7 @@
       <c r="L65" s="17"/>
       <c r="M65" s="17"/>
       <c r="N65" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B65, $C$2:$C$767, C65, $D$2:$D$767, D65, $E$2:$E$767, E65) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O65"/>
@@ -4384,7 +4362,7 @@
         <v>442</v>
       </c>
       <c r="N66" s="28" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B66, $C$2:$C$767, C66, $D$2:$D$767, D66, $E$2:$E$767, E66) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N66:N129" si="1">IF(COUNTIFS( $B$2:$B$767, B66, $C$2:$C$767, C66, $D$2:$D$767, D66, $E$2:$E$767, E66) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
       <c r="O66"/>
@@ -4423,7 +4401,7 @@
       <c r="L67" s="17"/>
       <c r="M67" s="17"/>
       <c r="N67" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B67, $C$2:$C$767, C67, $D$2:$D$767, D67, $E$2:$E$767, E67) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O67"/>
@@ -4464,7 +4442,7 @@
       <c r="L68" s="17"/>
       <c r="M68" s="17"/>
       <c r="N68" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B68, $C$2:$C$767, C68, $D$2:$D$767, D68, $E$2:$E$767, E68) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O68"/>
@@ -4503,7 +4481,7 @@
       <c r="L69" s="17"/>
       <c r="M69" s="17"/>
       <c r="N69" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B69, $C$2:$C$767, C69, $D$2:$D$767, D69, $E$2:$E$767, E69) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O69"/>
@@ -4542,7 +4520,7 @@
       <c r="L70" s="17"/>
       <c r="M70" s="17"/>
       <c r="N70" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B70, $C$2:$C$767, C70, $D$2:$D$767, D70, $E$2:$E$767, E70) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O70"/>
@@ -4581,7 +4559,7 @@
       <c r="L71" s="17"/>
       <c r="M71" s="17"/>
       <c r="N71" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B71, $C$2:$C$767, C71, $D$2:$D$767, D71, $E$2:$E$767, E71) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O71"/>
@@ -4620,7 +4598,7 @@
       <c r="L72" s="17"/>
       <c r="M72" s="17"/>
       <c r="N72" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B72, $C$2:$C$767, C72, $D$2:$D$767, D72, $E$2:$E$767, E72) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O72"/>
@@ -4659,7 +4637,7 @@
       <c r="L73" s="17"/>
       <c r="M73" s="17"/>
       <c r="N73" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B73, $C$2:$C$767, C73, $D$2:$D$767, D73, $E$2:$E$767, E73) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O73"/>
@@ -4698,7 +4676,7 @@
       <c r="L74" s="17"/>
       <c r="M74" s="17"/>
       <c r="N74" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B74, $C$2:$C$767, C74, $D$2:$D$767, D74, $E$2:$E$767, E74) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O74"/>
@@ -4737,7 +4715,7 @@
       <c r="L75" s="17"/>
       <c r="M75" s="17"/>
       <c r="N75" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B75, $C$2:$C$767, C75, $D$2:$D$767, D75, $E$2:$E$767, E75) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O75"/>
@@ -4776,7 +4754,7 @@
       <c r="L76" s="17"/>
       <c r="M76" s="17"/>
       <c r="N76" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B76, $C$2:$C$767, C76, $D$2:$D$767, D76, $E$2:$E$767, E76) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O76"/>
@@ -4815,7 +4793,7 @@
       <c r="L77" s="17"/>
       <c r="M77" s="17"/>
       <c r="N77" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B77, $C$2:$C$767, C77, $D$2:$D$767, D77, $E$2:$E$767, E77) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O77"/>
@@ -4854,7 +4832,7 @@
       <c r="L78" s="17"/>
       <c r="M78" s="17"/>
       <c r="N78" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B78, $C$2:$C$767, C78, $D$2:$D$767, D78, $E$2:$E$767, E78) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O78"/>
@@ -4902,7 +4880,7 @@
         <v>26810</v>
       </c>
       <c r="N79" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B79, $C$2:$C$767, C79, $D$2:$D$767, D79, $E$2:$E$767, E79) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O79" s="10"/>
@@ -4941,7 +4919,7 @@
       <c r="L80" s="17"/>
       <c r="M80" s="17"/>
       <c r="N80" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B80, $C$2:$C$767, C80, $D$2:$D$767, D80, $E$2:$E$767, E80) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O80"/>
@@ -4989,7 +4967,7 @@
         <v>275</v>
       </c>
       <c r="N81" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B81, $C$2:$C$767, C81, $D$2:$D$767, D81, $E$2:$E$767, E81) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
       <c r="O81" s="46" t="s">
@@ -5039,7 +5017,7 @@
         <v>225</v>
       </c>
       <c r="N82" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B82, $C$2:$C$767, C82, $D$2:$D$767, D82, $E$2:$E$767, E82) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
       <c r="O82" s="46" t="s">
@@ -5089,7 +5067,7 @@
         <v>300</v>
       </c>
       <c r="N83" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B83, $C$2:$C$767, C83, $D$2:$D$767, D83, $E$2:$E$767, E83) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5135,7 +5113,7 @@
         <v>1246</v>
       </c>
       <c r="N84" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B84, $C$2:$C$767, C84, $D$2:$D$767, D84, $E$2:$E$767, E84) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5181,7 +5159,7 @@
         <v>26710</v>
       </c>
       <c r="N85" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B85, $C$2:$C$767, C85, $D$2:$D$767, D85, $E$2:$E$767, E85) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O85" s="46" t="s">
@@ -5223,7 +5201,7 @@
       <c r="L86" s="17"/>
       <c r="M86" s="17"/>
       <c r="N86" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B86, $C$2:$C$767, C86, $D$2:$D$767, D86, $E$2:$E$767, E86) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O86"/>
@@ -5264,7 +5242,7 @@
       <c r="L87" s="18"/>
       <c r="M87" s="18"/>
       <c r="N87" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B87, $C$2:$C$767, C87, $D$2:$D$767, D87, $E$2:$E$767, E87) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O87" s="46" t="s">
@@ -5309,11 +5287,11 @@
         <v>19730.5</v>
       </c>
       <c r="M88" s="33">
-        <f>ABS((D88*E88)-L88)</f>
+        <f t="shared" ref="M88:M102" si="2">ABS((D88*E88)-L88)</f>
         <v>504.5</v>
       </c>
       <c r="N88" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B88, $C$2:$C$767, C88, $D$2:$D$767, D88, $E$2:$E$767, E88) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
       <c r="O88" s="46" t="s">
@@ -5359,11 +5337,11 @@
         <v>19690</v>
       </c>
       <c r="M89" s="33">
-        <f>ABS((D89*E89)-L89)</f>
+        <f t="shared" si="2"/>
         <v>545</v>
       </c>
       <c r="N89" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B89, $C$2:$C$767, C89, $D$2:$D$767, D89, $E$2:$E$767, E89) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
       <c r="O89" s="46" t="s">
@@ -5409,63 +5387,63 @@
         <v>35880</v>
       </c>
       <c r="M90" s="18">
-        <f>ABS((D90*E90)-L90)</f>
+        <f t="shared" si="2"/>
         <v>26610</v>
       </c>
       <c r="N90" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B90, $C$2:$C$767, C90, $D$2:$D$767, D90, $E$2:$E$767, E90) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O90" s="10"/>
       <c r="P90" s="10"/>
     </row>
-    <row r="91" spans="1:16" s="67" customFormat="1" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A91" s="61">
+    <row r="91" spans="1:16" customFormat="1" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A91" s="3">
         <v>46265.375694444447</v>
       </c>
-      <c r="B91" s="62" t="s">
+      <c r="B91" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C91" s="62" t="s">
-        <v>7</v>
-      </c>
-      <c r="D91" s="63">
+      <c r="C91" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D91" s="4">
         <v>5</v>
       </c>
-      <c r="E91" s="63">
+      <c r="E91" s="4">
         <v>1236</v>
       </c>
-      <c r="F91" s="63">
+      <c r="F91" s="4">
         <v>3.7086759520000001</v>
       </c>
-      <c r="G91" s="64" t="s">
+      <c r="G91" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="H91" s="65">
+      <c r="H91" s="5">
         <v>1191.8</v>
       </c>
-      <c r="I91" s="62" t="s">
-        <v>8</v>
-      </c>
-      <c r="J91" s="66" t="s">
+      <c r="I91" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J91" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="K91" s="66" t="s">
+      <c r="K91" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="L91" s="66">
+      <c r="L91" s="18">
         <v>5905</v>
       </c>
-      <c r="M91" s="66">
-        <f>ABS((D91*E91)-L91)</f>
+      <c r="M91" s="18">
+        <f t="shared" si="2"/>
         <v>275</v>
       </c>
-      <c r="N91" s="67" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B91, $C$2:$C$767, C91, $D$2:$D$767, D91, $E$2:$E$767, E91) &gt; 1, "Duplicate", "Unique")</f>
-        <v>Unique</v>
-      </c>
-      <c r="O91" s="68"/>
-      <c r="P91" s="68"/>
+      <c r="N91" t="str">
+        <f t="shared" si="1"/>
+        <v>Unique</v>
+      </c>
+      <c r="O91" s="10"/>
+      <c r="P91" s="10"/>
     </row>
     <row r="92" spans="1:16" customFormat="1" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="36">
@@ -5505,11 +5483,11 @@
         <v>3560</v>
       </c>
       <c r="M92" s="33">
-        <f>ABS((D92*E92)-L92)</f>
+        <f t="shared" si="2"/>
         <v>175</v>
       </c>
       <c r="N92" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B92, $C$2:$C$767, C92, $D$2:$D$767, D92, $E$2:$E$767, E92) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
       <c r="O92" s="46" t="s">
@@ -5554,11 +5532,11 @@
         <v>3510</v>
       </c>
       <c r="M93" s="33">
-        <f>ABS((D93*E93)-L93)</f>
+        <f t="shared" si="2"/>
         <v>225</v>
       </c>
       <c r="N93" s="34" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B93, $C$2:$C$767, C93, $D$2:$D$767, D93, $E$2:$E$767, E93) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
       <c r="O93" s="46" t="s">
@@ -5604,11 +5582,11 @@
         <v>8700</v>
       </c>
       <c r="M94" s="18">
-        <f>ABS((D94*E94)-L94)</f>
+        <f t="shared" si="2"/>
         <v>300</v>
       </c>
       <c r="N94" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B94, $C$2:$C$767, C94, $D$2:$D$767, D94, $E$2:$E$767, E94) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O94" s="10"/>
@@ -5652,11 +5630,11 @@
         <v>8220</v>
       </c>
       <c r="M95" s="18">
-        <f>ABS((D95*E95)-L95)</f>
+        <f t="shared" si="2"/>
         <v>360</v>
       </c>
       <c r="N95" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B95, $C$2:$C$767, C95, $D$2:$D$767, D95, $E$2:$E$767, E95) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O95" s="46" t="s">
@@ -5701,11 +5679,11 @@
         <v>20010</v>
       </c>
       <c r="M96" s="18">
-        <f>ABS((D96*E96)-L96)</f>
+        <f t="shared" si="2"/>
         <v>450</v>
       </c>
       <c r="N96" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B96, $C$2:$C$767, C96, $D$2:$D$767, D96, $E$2:$E$767, E96) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O96" s="10"/>
@@ -5749,11 +5727,11 @@
         <v>9170</v>
       </c>
       <c r="M97" s="33">
-        <f>ABS((D97*E97)-L97)</f>
+        <f t="shared" si="2"/>
         <v>200</v>
       </c>
       <c r="N97" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B97, $C$2:$C$767, C97, $D$2:$D$767, D97, $E$2:$E$767, E97) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O97" s="10"/>
@@ -5797,11 +5775,11 @@
         <v>8480</v>
       </c>
       <c r="M98" s="27">
-        <f>ABS((D98*E98)-L98)</f>
+        <f t="shared" si="2"/>
         <v>280</v>
       </c>
       <c r="N98" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B98, $C$2:$C$767, C98, $D$2:$D$767, D98, $E$2:$E$767, E98) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O98" s="46" t="s">
@@ -5847,11 +5825,11 @@
         <v>73800</v>
       </c>
       <c r="M99" s="18">
-        <f>ABS((D99*E99)-L99)</f>
+        <f t="shared" si="2"/>
         <v>48320</v>
       </c>
       <c r="N99" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B99, $C$2:$C$767, C99, $D$2:$D$767, D99, $E$2:$E$767, E99) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O99" s="46" t="s">
@@ -5897,11 +5875,11 @@
         <v>20260</v>
       </c>
       <c r="M100" s="18">
-        <f>ABS((D100*E100)-L100)</f>
+        <f t="shared" si="2"/>
         <v>300</v>
       </c>
       <c r="N100" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B100, $C$2:$C$767, C100, $D$2:$D$767, D100, $E$2:$E$767, E100) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O100"/>
@@ -5945,11 +5923,11 @@
         <v>9902</v>
       </c>
       <c r="M101" s="18">
-        <f>ABS((D101*E101)-L101)</f>
+        <f t="shared" si="2"/>
         <v>646</v>
       </c>
       <c r="N101" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B101, $C$2:$C$767, C101, $D$2:$D$767, D101, $E$2:$E$767, E101) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O101" s="46" t="s">
@@ -5995,11 +5973,11 @@
         <v>35880</v>
       </c>
       <c r="M102" s="18">
-        <f>ABS((D102*E102)-L102)</f>
+        <f t="shared" si="2"/>
         <v>26460</v>
       </c>
       <c r="N102" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B102, $C$2:$C$767, C102, $D$2:$D$767, D102, $E$2:$E$767, E102) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O102" s="10"/>
@@ -6035,7 +6013,7 @@
       </c>
       <c r="J103" s="40"/>
       <c r="N103" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B103, $C$2:$C$767, C103, $D$2:$D$767, D103, $E$2:$E$767, E103) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6069,7 +6047,7 @@
       </c>
       <c r="J104" s="40"/>
       <c r="N104" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B104, $C$2:$C$767, C104, $D$2:$D$767, D104, $E$2:$E$767, E104) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O104" s="46" t="s">
@@ -6119,7 +6097,7 @@
         <v>300</v>
       </c>
       <c r="N105" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B105, $C$2:$C$767, C105, $D$2:$D$767, D105, $E$2:$E$767, E105) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O105"/>
@@ -6167,7 +6145,7 @@
         <v>300.00000000000182</v>
       </c>
       <c r="N106" s="34" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B106, $C$2:$C$767, C106, $D$2:$D$767, D106, $E$2:$E$767, E106) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O106" s="46" t="s">
@@ -6217,7 +6195,7 @@
         <v>274</v>
       </c>
       <c r="N107" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B107, $C$2:$C$767, C107, $D$2:$D$767, D107, $E$2:$E$767, E107) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O107" s="46" t="s">
@@ -6267,7 +6245,7 @@
         <v>150</v>
       </c>
       <c r="N108" s="34" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B108, $C$2:$C$767, C108, $D$2:$D$767, D108, $E$2:$E$767, E108) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -6313,7 +6291,7 @@
         <v>250</v>
       </c>
       <c r="N109" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B109, $C$2:$C$767, C109, $D$2:$D$767, D109, $E$2:$E$767, E109) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Duplicate</v>
       </c>
       <c r="O109" s="10"/>
@@ -6349,7 +6327,7 @@
       </c>
       <c r="J110" s="40"/>
       <c r="N110" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B110, $C$2:$C$767, C110, $D$2:$D$767, D110, $E$2:$E$767, E110) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6391,11 +6369,11 @@
         <v>20070</v>
       </c>
       <c r="M111" s="18">
-        <f>ABS((D111*E111)-L111)</f>
+        <f t="shared" ref="M111:M123" si="3">ABS((D111*E111)-L111)</f>
         <v>810</v>
       </c>
       <c r="N111" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B111, $C$2:$C$767, C111, $D$2:$D$767, D111, $E$2:$E$767, E111) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6437,11 +6415,11 @@
         <v>15075</v>
       </c>
       <c r="M112" s="18">
-        <f>ABS((D112*E112)-L112)</f>
+        <f t="shared" si="3"/>
         <v>645</v>
       </c>
       <c r="N112" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B112, $C$2:$C$767, C112, $D$2:$D$767, D112, $E$2:$E$767, E112) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O112" s="46" t="s">
@@ -6486,11 +6464,11 @@
         <v>9170</v>
       </c>
       <c r="M113" s="33">
-        <f>ABS((D113*E113)-L113)</f>
+        <f t="shared" si="3"/>
         <v>300</v>
       </c>
       <c r="N113" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B113, $C$2:$C$767, C113, $D$2:$D$767, D113, $E$2:$E$767, E113) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O113" s="10"/>
@@ -6534,11 +6512,11 @@
         <v>8420</v>
       </c>
       <c r="M114" s="18">
-        <f>ABS((D114*E114)-L114)</f>
+        <f t="shared" si="3"/>
         <v>300</v>
       </c>
       <c r="N114" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B114, $C$2:$C$767, C114, $D$2:$D$767, D114, $E$2:$E$767, E114) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6580,11 +6558,11 @@
         <v>11320</v>
       </c>
       <c r="M115" s="18">
-        <f>ABS((D115*E115)-L115)</f>
+        <f t="shared" si="3"/>
         <v>400</v>
       </c>
       <c r="N115" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B115, $C$2:$C$767, C115, $D$2:$D$767, D115, $E$2:$E$767, E115) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6626,11 +6604,11 @@
         <v>3005</v>
       </c>
       <c r="M116" s="18">
-        <f>ABS((D116*E116)-L116)</f>
+        <f t="shared" si="3"/>
         <v>240</v>
       </c>
       <c r="N116" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B116, $C$2:$C$767, C116, $D$2:$D$767, D116, $E$2:$E$767, E116) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O116" s="10"/>
@@ -6674,11 +6652,11 @@
         <v>14100</v>
       </c>
       <c r="M117" s="18">
-        <f>ABS((D117*E117)-L117)</f>
+        <f t="shared" si="3"/>
         <v>500</v>
       </c>
       <c r="N117" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B117, $C$2:$C$767, C117, $D$2:$D$767, D117, $E$2:$E$767, E117) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O117" s="10"/>
@@ -6722,11 +6700,11 @@
         <v>73800</v>
       </c>
       <c r="M118" s="18">
-        <f>ABS((D118*E118)-L118)</f>
+        <f t="shared" si="3"/>
         <v>47900</v>
       </c>
       <c r="N118" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B118, $C$2:$C$767, C118, $D$2:$D$767, D118, $E$2:$E$767, E118) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O118" s="46" t="s">
@@ -6771,11 +6749,11 @@
         <v>18960</v>
       </c>
       <c r="M119" s="18">
-        <f>ABS((D119*E119)-L119)</f>
+        <f t="shared" si="3"/>
         <v>816</v>
       </c>
       <c r="N119" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B119, $C$2:$C$767, C119, $D$2:$D$767, D119, $E$2:$E$767, E119) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6817,11 +6795,11 @@
         <v>3300</v>
       </c>
       <c r="M120" s="18">
-        <f>ABS((D120*E120)-L120)</f>
+        <f t="shared" si="3"/>
         <v>250</v>
       </c>
       <c r="N120" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B120, $C$2:$C$767, C120, $D$2:$D$767, D120, $E$2:$E$767, E120) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6863,11 +6841,11 @@
         <v>25300</v>
       </c>
       <c r="M121" s="18">
-        <f>ABS((D121*E121)-L121)</f>
+        <f t="shared" si="3"/>
         <v>650</v>
       </c>
       <c r="N121" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B121, $C$2:$C$767, C121, $D$2:$D$767, D121, $E$2:$E$767, E121) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O121" s="46" t="s">
@@ -6912,11 +6890,11 @@
         <v>12480</v>
       </c>
       <c r="M122" s="18">
-        <f>ABS((D122*E122)-L122)</f>
+        <f t="shared" si="3"/>
         <v>495</v>
       </c>
       <c r="N122" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B122, $C$2:$C$767, C122, $D$2:$D$767, D122, $E$2:$E$767, E122) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O122" s="46" t="s">
@@ -6961,11 +6939,11 @@
         <v>32200</v>
       </c>
       <c r="M123" s="18">
-        <f>ABS((D123*E123)-L123)</f>
+        <f t="shared" si="3"/>
         <v>1200</v>
       </c>
       <c r="N123" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B123, $C$2:$C$767, C123, $D$2:$D$767, D123, $E$2:$E$767, E123) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6999,7 +6977,7 @@
       </c>
       <c r="J124" s="40"/>
       <c r="N124" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B124, $C$2:$C$767, C124, $D$2:$D$767, D124, $E$2:$E$767, E124) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O124" s="25"/>
@@ -7042,11 +7020,11 @@
         <v>26109.000000000004</v>
       </c>
       <c r="M125" s="33">
-        <f>ABS((D125*E125)-L125)</f>
+        <f t="shared" ref="M125:M130" si="4">ABS((D125*E125)-L125)</f>
         <v>710.99999999999636</v>
       </c>
       <c r="N125" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B125, $C$2:$C$767, C125, $D$2:$D$767, D125, $E$2:$E$767, E125) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O125" s="46" t="s">
@@ -7092,11 +7070,11 @@
         <v>8570</v>
       </c>
       <c r="M126" s="33">
-        <f>ABS((D126*E126)-L126)</f>
+        <f t="shared" si="4"/>
         <v>650</v>
       </c>
       <c r="N126" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B126, $C$2:$C$767, C126, $D$2:$D$767, D126, $E$2:$E$767, E126) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O126" s="46" t="s">
@@ -7141,11 +7119,11 @@
         <v>9270</v>
       </c>
       <c r="M127" s="18">
-        <f>ABS((D127*E127)-L127)</f>
+        <f t="shared" si="4"/>
         <v>300</v>
       </c>
       <c r="N127" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B127, $C$2:$C$767, C127, $D$2:$D$767, D127, $E$2:$E$767, E127) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="P127" s="19"/>
@@ -7188,11 +7166,11 @@
         <v>10300</v>
       </c>
       <c r="M128" s="18">
-        <f>ABS((D128*E128)-L128)</f>
+        <f t="shared" si="4"/>
         <v>300</v>
       </c>
       <c r="N128" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B128, $C$2:$C$767, C128, $D$2:$D$767, D128, $E$2:$E$767, E128) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
       <c r="O128" s="10"/>
@@ -7236,11 +7214,11 @@
         <v>14200</v>
       </c>
       <c r="M129" s="18">
-        <f>ABS((D129*E129)-L129)</f>
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
       <c r="N129" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B129, $C$2:$C$767, C129, $D$2:$D$767, D129, $E$2:$E$767, E129) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7282,11 +7260,11 @@
         <v>25780</v>
       </c>
       <c r="M130" s="18">
-        <f>ABS((D130*E130)-L130)</f>
+        <f t="shared" si="4"/>
         <v>300</v>
       </c>
       <c r="N130" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B130, $C$2:$C$767, C130, $D$2:$D$767, D130, $E$2:$E$767, E130) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N130:N193" si="5">IF(COUNTIFS( $B$2:$B$767, B130, $C$2:$C$767, C130, $D$2:$D$767, D130, $E$2:$E$767, E130) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
       <c r="O130" s="46" t="s">
@@ -7326,7 +7304,7 @@
         <v>117</v>
       </c>
       <c r="N131" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B131, $C$2:$C$767, C131, $D$2:$D$767, D131, $E$2:$E$767, E131) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7372,7 +7350,7 @@
         <v>651</v>
       </c>
       <c r="N132" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B132, $C$2:$C$767, C132, $D$2:$D$767, D132, $E$2:$E$767, E132) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7418,7 +7396,7 @@
         <v>300</v>
       </c>
       <c r="N133" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B133, $C$2:$C$767, C133, $D$2:$D$767, D133, $E$2:$E$767, E133) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7464,7 +7442,7 @@
         <v>650</v>
       </c>
       <c r="N134" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B134, $C$2:$C$767, C134, $D$2:$D$767, D134, $E$2:$E$767, E134) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O134"/>
@@ -7512,7 +7490,7 @@
         <v>270</v>
       </c>
       <c r="N135" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B135, $C$2:$C$767, C135, $D$2:$D$767, D135, $E$2:$E$767, E135) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O135" s="47" t="s">
@@ -7549,7 +7527,7 @@
       </c>
       <c r="J136" s="40"/>
       <c r="N136" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B136, $C$2:$C$767, C136, $D$2:$D$767, D136, $E$2:$E$767, E136) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7595,7 +7573,7 @@
         <v>880</v>
       </c>
       <c r="N137" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B137, $C$2:$C$767, C137, $D$2:$D$767, D137, $E$2:$E$767, E137) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O137" s="46" t="s">
@@ -7634,7 +7612,7 @@
         <v>118</v>
       </c>
       <c r="N138" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B138, $C$2:$C$767, C138, $D$2:$D$767, D138, $E$2:$E$767, E138) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7676,11 +7654,11 @@
         <v>4080</v>
       </c>
       <c r="M139" s="18">
-        <f>ABS((D139*E139)-L139)</f>
+        <f t="shared" ref="M139:M144" si="6">ABS((D139*E139)-L139)</f>
         <v>300</v>
       </c>
       <c r="N139" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B139, $C$2:$C$767, C139, $D$2:$D$767, D139, $E$2:$E$767, E139) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7722,11 +7700,11 @@
         <v>5370</v>
       </c>
       <c r="M140" s="18">
-        <f>ABS((D140*E140)-L140)</f>
+        <f t="shared" si="6"/>
         <v>320</v>
       </c>
       <c r="N140" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B140, $C$2:$C$767, C140, $D$2:$D$767, D140, $E$2:$E$767, E140) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7768,11 +7746,11 @@
         <v>16580</v>
       </c>
       <c r="M141" s="54">
-        <f>ABS((D141*E141)-L141)</f>
+        <f t="shared" si="6"/>
         <v>750</v>
       </c>
       <c r="N141" s="25" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B141, $C$2:$C$767, C141, $D$2:$D$767, D141, $E$2:$E$767, E141) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O141" s="25"/>
@@ -7818,11 +7796,11 @@
         <v>10410</v>
       </c>
       <c r="M142" s="18">
-        <f>ABS((D142*E142)-L142)</f>
+        <f t="shared" si="6"/>
         <v>300</v>
       </c>
       <c r="N142" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B142, $C$2:$C$767, C142, $D$2:$D$767, D142, $E$2:$E$767, E142) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O142" s="35"/>
@@ -7865,11 +7843,11 @@
         <v>73800</v>
       </c>
       <c r="M143" s="18">
-        <f>ABS((D143*E143)-L143)</f>
+        <f t="shared" si="6"/>
         <v>47480</v>
       </c>
       <c r="N143" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B143, $C$2:$C$767, C143, $D$2:$D$767, D143, $E$2:$E$767, E143) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7911,11 +7889,11 @@
         <v>12510</v>
       </c>
       <c r="M144" s="18">
-        <f>ABS((D144*E144)-L144)</f>
+        <f t="shared" si="6"/>
         <v>290</v>
       </c>
       <c r="N144" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B144, $C$2:$C$767, C144, $D$2:$D$767, D144, $E$2:$E$767, E144) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7949,7 +7927,7 @@
       </c>
       <c r="J145" s="40"/>
       <c r="N145" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B145, $C$2:$C$767, C145, $D$2:$D$767, D145, $E$2:$E$767, E145) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7991,11 +7969,11 @@
         <v>32900</v>
       </c>
       <c r="M146" s="33">
-        <f>ABS((D146*E146)-L146)</f>
+        <f t="shared" ref="M146:M158" si="7">ABS((D146*E146)-L146)</f>
         <v>1000</v>
       </c>
       <c r="N146" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B146, $C$2:$C$767, C146, $D$2:$D$767, D146, $E$2:$E$767, E146) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Duplicate</v>
       </c>
       <c r="O146" s="26"/>
@@ -8038,11 +8016,11 @@
         <v>33200</v>
       </c>
       <c r="M147" s="33">
-        <f>ABS((D147*E147)-L147)</f>
+        <f t="shared" si="7"/>
         <v>700</v>
       </c>
       <c r="N147" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B147, $C$2:$C$767, C147, $D$2:$D$767, D147, $E$2:$E$767, E147) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -8084,11 +8062,11 @@
         <v>26020</v>
       </c>
       <c r="M148" s="18">
-        <f>ABS((D148*E148)-L148)</f>
+        <f t="shared" si="7"/>
         <v>340</v>
       </c>
       <c r="N148" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B148, $C$2:$C$767, C148, $D$2:$D$767, D148, $E$2:$E$767, E148) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O148" s="10"/>
@@ -8132,11 +8110,11 @@
         <v>11660</v>
       </c>
       <c r="M149" s="18">
-        <f>ABS((D149*E149)-L149)</f>
+        <f t="shared" si="7"/>
         <v>300</v>
       </c>
       <c r="N149" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B149, $C$2:$C$767, C149, $D$2:$D$767, D149, $E$2:$E$767, E149) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O149" s="46" t="s">
@@ -8181,11 +8159,11 @@
         <v>14400</v>
       </c>
       <c r="M150" s="18">
-        <f>ABS((D150*E150)-L150)</f>
+        <f t="shared" si="7"/>
         <v>500</v>
       </c>
       <c r="N150" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B150, $C$2:$C$767, C150, $D$2:$D$767, D150, $E$2:$E$767, E150) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8227,11 +8205,11 @@
         <v>5180</v>
       </c>
       <c r="M151" s="27">
-        <f>ABS((D151*E151)-L151)</f>
+        <f t="shared" si="7"/>
         <v>268</v>
       </c>
       <c r="N151" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B151, $C$2:$C$767, C151, $D$2:$D$767, D151, $E$2:$E$767, E151) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8273,11 +8251,11 @@
         <v>18140</v>
       </c>
       <c r="M152" s="27">
-        <f>ABS((D152*E152)-L152)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="N152" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B152, $C$2:$C$767, C152, $D$2:$D$767, D152, $E$2:$E$767, E152) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O152" s="46" t="s">
@@ -8322,11 +8300,11 @@
         <v>26180</v>
       </c>
       <c r="M153" s="18">
-        <f>ABS((D153*E153)-L153)</f>
+        <f t="shared" si="7"/>
         <v>300</v>
       </c>
       <c r="N153" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B153, $C$2:$C$767, C153, $D$2:$D$767, D153, $E$2:$E$767, E153) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O153" s="10"/>
@@ -8370,11 +8348,11 @@
         <v>16755</v>
       </c>
       <c r="M154" s="18">
-        <f>ABS((D154*E154)-L154)</f>
+        <f t="shared" si="7"/>
         <v>295</v>
       </c>
       <c r="N154" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B154, $C$2:$C$767, C154, $D$2:$D$767, D154, $E$2:$E$767, E154) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8416,11 +8394,11 @@
         <v>8049</v>
       </c>
       <c r="M155" s="18">
-        <f>ABS((D155*E155)-L155)</f>
+        <f t="shared" si="7"/>
         <v>800</v>
       </c>
       <c r="N155" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B155, $C$2:$C$767, C155, $D$2:$D$767, D155, $E$2:$E$767, E155) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8462,11 +8440,11 @@
         <v>10510</v>
       </c>
       <c r="M156" s="18">
-        <f>ABS((D156*E156)-L156)</f>
+        <f t="shared" si="7"/>
         <v>300</v>
       </c>
       <c r="N156" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B156, $C$2:$C$767, C156, $D$2:$D$767, D156, $E$2:$E$767, E156) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8508,11 +8486,11 @@
         <v>18800</v>
       </c>
       <c r="M157" s="18">
-        <f>ABS((D157*E157)-L157)</f>
+        <f t="shared" si="7"/>
         <v>500</v>
       </c>
       <c r="N157" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B157, $C$2:$C$767, C157, $D$2:$D$767, D157, $E$2:$E$767, E157) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O157" s="47" t="s">
@@ -8557,11 +8535,11 @@
         <v>9470</v>
       </c>
       <c r="M158" s="18">
-        <f>ABS((D158*E158)-L158)</f>
+        <f t="shared" si="7"/>
         <v>300</v>
       </c>
       <c r="N158" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B158, $C$2:$C$767, C158, $D$2:$D$767, D158, $E$2:$E$767, E158) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8597,7 +8575,7 @@
         <v>118</v>
       </c>
       <c r="N159" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B159, $C$2:$C$767, C159, $D$2:$D$767, D159, $E$2:$E$767, E159) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8643,7 +8621,7 @@
         <v>300</v>
       </c>
       <c r="N160" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B160, $C$2:$C$767, C160, $D$2:$D$767, D160, $E$2:$E$767, E160) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8682,7 +8660,7 @@
       <c r="L161" s="54"/>
       <c r="M161" s="54"/>
       <c r="N161" s="25" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B161, $C$2:$C$767, C161, $D$2:$D$767, D161, $E$2:$E$767, E161) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O161" s="25"/>
@@ -8728,11 +8706,11 @@
         <v>12600</v>
       </c>
       <c r="M162" s="18">
-        <f>ABS((D162*E162)-L162)</f>
+        <f t="shared" ref="M162:M168" si="8">ABS((D162*E162)-L162)</f>
         <v>360</v>
       </c>
       <c r="N162" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B162, $C$2:$C$767, C162, $D$2:$D$767, D162, $E$2:$E$767, E162) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8774,11 +8752,11 @@
         <v>3400</v>
       </c>
       <c r="M163" s="18">
-        <f>ABS((D163*E163)-L163)</f>
+        <f t="shared" si="8"/>
         <v>250</v>
       </c>
       <c r="N163" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B163, $C$2:$C$767, C163, $D$2:$D$767, D163, $E$2:$E$767, E163) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8820,11 +8798,11 @@
         <v>7578</v>
       </c>
       <c r="M164" s="33">
-        <f>ABS((D164*E164)-L164)</f>
+        <f t="shared" si="8"/>
         <v>294</v>
       </c>
       <c r="N164" s="34" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B164, $C$2:$C$767, C164, $D$2:$D$767, D164, $E$2:$E$767, E164) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Duplicate</v>
       </c>
       <c r="O164" s="10"/>
@@ -8868,40 +8846,40 @@
         <v>7578</v>
       </c>
       <c r="M165" s="33">
-        <f>ABS((D165*E165)-L165)</f>
+        <f t="shared" si="8"/>
         <v>294</v>
       </c>
       <c r="N165" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B165, $C$2:$C$767, C165, $D$2:$D$767, D165, $E$2:$E$767, E165) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Duplicate</v>
       </c>
     </row>
     <row r="166" spans="1:16" s="35" customFormat="1" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A166" s="69">
+      <c r="A166" s="61">
         <v>46267.424305555556</v>
       </c>
-      <c r="B166" s="70" t="s">
+      <c r="B166" s="62" t="s">
         <v>53</v>
       </c>
-      <c r="C166" s="70" t="s">
-        <v>7</v>
-      </c>
-      <c r="D166" s="71">
+      <c r="C166" s="62" t="s">
+        <v>7</v>
+      </c>
+      <c r="D166" s="63">
         <v>2</v>
       </c>
-      <c r="E166" s="71">
+      <c r="E166" s="63">
         <v>2624</v>
       </c>
-      <c r="F166" s="71">
+      <c r="F166" s="63">
         <v>8.9746251919999995</v>
       </c>
-      <c r="G166" s="72" t="s">
+      <c r="G166" s="64" t="s">
         <v>54</v>
       </c>
-      <c r="H166" s="73">
+      <c r="H166" s="65">
         <v>2407.9</v>
       </c>
-      <c r="I166" s="70" t="s">
+      <c r="I166" s="62" t="s">
         <v>8</v>
       </c>
       <c r="J166" s="33" t="s">
@@ -8914,40 +8892,40 @@
         <v>4968</v>
       </c>
       <c r="M166" s="33">
-        <f>ABS((D166*E166)-L166)</f>
+        <f t="shared" si="8"/>
         <v>280</v>
       </c>
       <c r="N166" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B166, $C$2:$C$767, C166, $D$2:$D$767, D166, $E$2:$E$767, E166) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="167" spans="1:16" s="35" customFormat="1" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A167" s="69">
+      <c r="A167" s="61">
         <v>46272.451388888891</v>
       </c>
-      <c r="B167" s="70" t="s">
+      <c r="B167" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C167" s="70" t="s">
-        <v>7</v>
-      </c>
-      <c r="D167" s="71">
+      <c r="C167" s="62" t="s">
+        <v>7</v>
+      </c>
+      <c r="D167" s="63">
         <v>5</v>
       </c>
-      <c r="E167" s="71">
+      <c r="E167" s="63">
         <v>1894</v>
       </c>
-      <c r="F167" s="71">
+      <c r="F167" s="63">
         <v>8.975834292</v>
       </c>
-      <c r="G167" s="72" t="s">
+      <c r="G167" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="H167" s="73">
+      <c r="H167" s="65">
         <v>1738</v>
       </c>
-      <c r="I167" s="70" t="s">
+      <c r="I167" s="62" t="s">
         <v>8</v>
       </c>
       <c r="J167" s="35" t="s">
@@ -8960,40 +8938,40 @@
         <v>8820</v>
       </c>
       <c r="M167" s="33">
-        <f>ABS((D167*E167)-L167)</f>
+        <f t="shared" si="8"/>
         <v>650</v>
       </c>
       <c r="N167" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B167, $C$2:$C$767, C167, $D$2:$D$767, D167, $E$2:$E$767, E167) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
     <row r="168" spans="1:16" s="35" customFormat="1" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A168" s="69">
+      <c r="A168" s="61">
         <v>46272.390972222223</v>
       </c>
-      <c r="B168" s="70" t="s">
+      <c r="B168" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C168" s="70" t="s">
-        <v>7</v>
-      </c>
-      <c r="D168" s="71">
+      <c r="C168" s="62" t="s">
+        <v>7</v>
+      </c>
+      <c r="D168" s="63">
         <v>20</v>
       </c>
-      <c r="E168" s="71">
+      <c r="E168" s="63">
         <v>1894</v>
       </c>
-      <c r="F168" s="71">
+      <c r="F168" s="63">
         <v>8.975834292</v>
       </c>
-      <c r="G168" s="72" t="s">
+      <c r="G168" s="64" t="s">
         <v>91</v>
       </c>
-      <c r="H168" s="73">
+      <c r="H168" s="65">
         <v>1738</v>
       </c>
-      <c r="I168" s="70" t="s">
+      <c r="I168" s="62" t="s">
         <v>8</v>
       </c>
       <c r="J168" s="35" t="s">
@@ -9006,11 +8984,11 @@
         <v>36946</v>
       </c>
       <c r="M168" s="33">
-        <f>ABS((D168*E168)-L168)</f>
+        <f t="shared" si="8"/>
         <v>934</v>
       </c>
       <c r="N168" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B168, $C$2:$C$767, C168, $D$2:$D$767, D168, $E$2:$E$767, E168) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9051,7 +9029,7 @@
       <c r="L169" s="17"/>
       <c r="M169" s="17"/>
       <c r="N169" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B169, $C$2:$C$767, C169, $D$2:$D$767, D169, $E$2:$E$767, E169) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9062,7 +9040,7 @@
       <c r="B170" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="C170" s="74" t="s">
+      <c r="C170" s="66" t="s">
         <v>7</v>
       </c>
       <c r="D170" s="8">
@@ -9085,7 +9063,7 @@
       </c>
       <c r="J170" s="40"/>
       <c r="N170" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B170, $C$2:$C$767, C170, $D$2:$D$767, D170, $E$2:$E$767, E170) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O170" s="35"/>
@@ -9132,7 +9110,7 @@
         <v>500</v>
       </c>
       <c r="N171" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B171, $C$2:$C$767, C171, $D$2:$D$767, D171, $E$2:$E$767, E171) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9178,7 +9156,7 @@
         <v>450</v>
       </c>
       <c r="N172" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B172, $C$2:$C$767, C172, $D$2:$D$767, D172, $E$2:$E$767, E172) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9214,7 +9192,7 @@
         <v>118</v>
       </c>
       <c r="N173" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B173, $C$2:$C$767, C173, $D$2:$D$767, D173, $E$2:$E$767, E173) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9260,7 +9238,7 @@
         <v>300</v>
       </c>
       <c r="N174" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B174, $C$2:$C$767, C174, $D$2:$D$767, D174, $E$2:$E$767, E174) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9306,7 +9284,7 @@
         <v>650</v>
       </c>
       <c r="N175" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B175, $C$2:$C$767, C175, $D$2:$D$767, D175, $E$2:$E$767, E175) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O175" s="46" t="s">
@@ -9346,7 +9324,7 @@
         <v>117</v>
       </c>
       <c r="N176" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B176, $C$2:$C$767, C176, $D$2:$D$767, D176, $E$2:$E$767, E176) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9392,7 +9370,7 @@
         <v>250</v>
       </c>
       <c r="N177" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B177, $C$2:$C$767, C177, $D$2:$D$767, D177, $E$2:$E$767, E177) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9438,7 +9416,7 @@
         <v>300</v>
       </c>
       <c r="N178" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B178, $C$2:$C$767, C178, $D$2:$D$767, D178, $E$2:$E$767, E178) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9475,7 +9453,7 @@
       <c r="L179" s="18"/>
       <c r="M179" s="18"/>
       <c r="N179" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B179, $C$2:$C$767, C179, $D$2:$D$767, D179, $E$2:$E$767, E179) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O179" s="10"/>
@@ -9523,7 +9501,7 @@
         <v>250</v>
       </c>
       <c r="N180" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B180, $C$2:$C$767, C180, $D$2:$D$767, D180, $E$2:$E$767, E180) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O180" s="10"/>
@@ -9561,7 +9539,7 @@
         <v>156</v>
       </c>
       <c r="N181" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B181, $C$2:$C$767, C181, $D$2:$D$767, D181, $E$2:$E$767, E181) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9597,7 +9575,7 @@
         <v>118</v>
       </c>
       <c r="N182" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B182, $C$2:$C$767, C182, $D$2:$D$767, D182, $E$2:$E$767, E182) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O182" s="46" t="s">
@@ -9634,7 +9612,7 @@
       </c>
       <c r="J183" s="21"/>
       <c r="N183" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B183, $C$2:$C$767, C183, $D$2:$D$767, D183, $E$2:$E$767, E183) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9680,7 +9658,7 @@
         <v>300</v>
       </c>
       <c r="N184" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B184, $C$2:$C$767, C184, $D$2:$D$767, D184, $E$2:$E$767, E184) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O184" s="46" t="s">
@@ -9730,7 +9708,7 @@
         <v>501</v>
       </c>
       <c r="N185" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B185, $C$2:$C$767, C185, $D$2:$D$767, D185, $E$2:$E$767, E185) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O185" s="46" t="s">
@@ -9770,7 +9748,7 @@
         <v>117</v>
       </c>
       <c r="N186" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B186, $C$2:$C$767, C186, $D$2:$D$767, D186, $E$2:$E$767, E186) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9816,7 +9794,7 @@
         <v>700</v>
       </c>
       <c r="N187" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B187, $C$2:$C$767, C187, $D$2:$D$767, D187, $E$2:$E$767, E187) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O187" s="35"/>
@@ -9863,7 +9841,7 @@
         <v>250</v>
       </c>
       <c r="N188" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B188, $C$2:$C$767, C188, $D$2:$D$767, D188, $E$2:$E$767, E188) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="P188" s="35"/>
@@ -9910,7 +9888,7 @@
         <v>1000</v>
       </c>
       <c r="N189" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B189, $C$2:$C$767, C189, $D$2:$D$767, D189, $E$2:$E$767, E189) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="P189" s="35"/>
@@ -9957,7 +9935,7 @@
         <v>320</v>
       </c>
       <c r="N190" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B190, $C$2:$C$767, C190, $D$2:$D$767, D190, $E$2:$E$767, E190) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10003,7 +9981,7 @@
         <v>448</v>
       </c>
       <c r="N191" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B191, $C$2:$C$767, C191, $D$2:$D$767, D191, $E$2:$E$767, E191) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10039,7 +10017,7 @@
         <v>117</v>
       </c>
       <c r="N192" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B192, $C$2:$C$767, C192, $D$2:$D$767, D192, $E$2:$E$767, E192) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10085,7 +10063,7 @@
         <v>300</v>
       </c>
       <c r="N193" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B193, $C$2:$C$767, C193, $D$2:$D$767, D193, $E$2:$E$767, E193) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="5"/>
         <v>Unique</v>
       </c>
       <c r="O193" s="10"/>
@@ -10121,7 +10099,7 @@
       </c>
       <c r="J194" s="40"/>
       <c r="N194" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B194, $C$2:$C$767, C194, $D$2:$D$767, D194, $E$2:$E$767, E194) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N194:N257" si="9">IF(COUNTIFS( $B$2:$B$767, B194, $C$2:$C$767, C194, $D$2:$D$767, D194, $E$2:$E$767, E194) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -10167,7 +10145,7 @@
         <v>300</v>
       </c>
       <c r="N195" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B195, $C$2:$C$767, C195, $D$2:$D$767, D195, $E$2:$E$767, E195) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P195" s="26"/>
@@ -10214,7 +10192,7 @@
         <v>400</v>
       </c>
       <c r="N196" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B196, $C$2:$C$767, C196, $D$2:$D$767, D196, $E$2:$E$767, E196) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10253,7 +10231,7 @@
         <v>144</v>
       </c>
       <c r="N197" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B197, $C$2:$C$767, C197, $D$2:$D$767, D197, $E$2:$E$767, E197) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10299,7 +10277,7 @@
         <v>140</v>
       </c>
       <c r="N198" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B198, $C$2:$C$767, C198, $D$2:$D$767, D198, $E$2:$E$767, E198) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
       <c r="O198" s="10"/>
@@ -10346,7 +10324,7 @@
         <v>300</v>
       </c>
       <c r="N199" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B199, $C$2:$C$767, C199, $D$2:$D$767, D199, $E$2:$E$767, E199) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
       <c r="O199" s="10"/>
@@ -10384,7 +10362,7 @@
         <v>117</v>
       </c>
       <c r="N200" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B200, $C$2:$C$767, C200, $D$2:$D$767, D200, $E$2:$E$767, E200) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10418,7 +10396,7 @@
       </c>
       <c r="J201" s="40"/>
       <c r="N201" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B201, $C$2:$C$767, C201, $D$2:$D$767, D201, $E$2:$E$767, E201) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P201" s="35"/>
@@ -10465,7 +10443,7 @@
         <v>300</v>
       </c>
       <c r="N202" s="34" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B202, $C$2:$C$767, C202, $D$2:$D$767, D202, $E$2:$E$767, E202) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O202" s="35"/>
@@ -10512,7 +10490,7 @@
         <v>253</v>
       </c>
       <c r="N203" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B203, $C$2:$C$767, C203, $D$2:$D$767, D203, $E$2:$E$767, E203) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O203" s="35"/>
@@ -10559,7 +10537,7 @@
         <v>260</v>
       </c>
       <c r="N204" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B204, $C$2:$C$767, C204, $D$2:$D$767, D204, $E$2:$E$767, E204) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10595,7 +10573,7 @@
         <v>198</v>
       </c>
       <c r="N205" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B205, $C$2:$C$767, C205, $D$2:$D$767, D205, $E$2:$E$767, E205) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10631,7 +10609,7 @@
         <v>117</v>
       </c>
       <c r="N206" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B206, $C$2:$C$767, C206, $D$2:$D$767, D206, $E$2:$E$767, E206) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10667,7 +10645,7 @@
         <v>118</v>
       </c>
       <c r="N207" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B207, $C$2:$C$767, C207, $D$2:$D$767, D207, $E$2:$E$767, E207) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10713,7 +10691,7 @@
         <v>800</v>
       </c>
       <c r="N208" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B208, $C$2:$C$767, C208, $D$2:$D$767, D208, $E$2:$E$767, E208) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10759,7 +10737,7 @@
         <v>300</v>
       </c>
       <c r="N209" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B209, $C$2:$C$767, C209, $D$2:$D$767, D209, $E$2:$E$767, E209) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10805,7 +10783,7 @@
         <v>188</v>
       </c>
       <c r="N210" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B210, $C$2:$C$767, C210, $D$2:$D$767, D210, $E$2:$E$767, E210) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P210" s="35"/>
@@ -10842,7 +10820,7 @@
         <v>55</v>
       </c>
       <c r="N211" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B211, $C$2:$C$767, C211, $D$2:$D$767, D211, $E$2:$E$767, E211) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10881,7 +10859,7 @@
         <v>145</v>
       </c>
       <c r="N212" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B212, $C$2:$C$767, C212, $D$2:$D$767, D212, $E$2:$E$767, E212) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10927,7 +10905,7 @@
         <v>940</v>
       </c>
       <c r="N213" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B213, $C$2:$C$767, C213, $D$2:$D$767, D213, $E$2:$E$767, E213) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10973,7 +10951,7 @@
         <v>450</v>
       </c>
       <c r="N214" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B214, $C$2:$C$767, C214, $D$2:$D$767, D214, $E$2:$E$767, E214) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11009,7 +10987,7 @@
         <v>118</v>
       </c>
       <c r="N215" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B215, $C$2:$C$767, C215, $D$2:$D$767, D215, $E$2:$E$767, E215) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11055,7 +11033,7 @@
         <v>300</v>
       </c>
       <c r="N216" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B216, $C$2:$C$767, C216, $D$2:$D$767, D216, $E$2:$E$767, E216) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11091,7 +11069,7 @@
         <v>118</v>
       </c>
       <c r="N217" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B217, $C$2:$C$767, C217, $D$2:$D$767, D217, $E$2:$E$767, E217) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11137,7 +11115,7 @@
         <v>370</v>
       </c>
       <c r="N218" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B218, $C$2:$C$767, C218, $D$2:$D$767, D218, $E$2:$E$767, E218) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P218" s="35"/>
@@ -11184,7 +11162,7 @@
         <v>527.5</v>
       </c>
       <c r="N219" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B219, $C$2:$C$767, C219, $D$2:$D$767, D219, $E$2:$E$767, E219) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O219" s="35"/>
@@ -11227,7 +11205,7 @@
       <c r="L220" s="33"/>
       <c r="M220" s="33"/>
       <c r="N220" s="35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B220, $C$2:$C$767, C220, $D$2:$D$767, D220, $E$2:$E$767, E220) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O220" s="35"/>
@@ -11266,7 +11244,7 @@
       <c r="L221" s="18"/>
       <c r="M221" s="18"/>
       <c r="N221" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B221, $C$2:$C$767, C221, $D$2:$D$767, D221, $E$2:$E$767, E221) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O221" s="10"/>
@@ -11314,7 +11292,7 @@
         <v>1800</v>
       </c>
       <c r="N222" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B222, $C$2:$C$767, C222, $D$2:$D$767, D222, $E$2:$E$767, E222) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11348,7 +11326,7 @@
       </c>
       <c r="J223" s="40"/>
       <c r="N223" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B223, $C$2:$C$767, C223, $D$2:$D$767, D223, $E$2:$E$767, E223) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11394,7 +11372,7 @@
         <v>650</v>
       </c>
       <c r="N224" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B224, $C$2:$C$767, C224, $D$2:$D$767, D224, $E$2:$E$767, E224) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O224" s="35"/>
@@ -11441,7 +11419,7 @@
         <v>500</v>
       </c>
       <c r="N225" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B225, $C$2:$C$767, C225, $D$2:$D$767, D225, $E$2:$E$767, E225) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O225" s="46" t="s">
@@ -11483,7 +11461,7 @@
       <c r="L226" s="18"/>
       <c r="M226" s="18"/>
       <c r="N226" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B226, $C$2:$C$767, C226, $D$2:$D$767, D226, $E$2:$E$767, E226) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P226" s="10"/>
@@ -11520,7 +11498,7 @@
         <v>117</v>
       </c>
       <c r="N227" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B227, $C$2:$C$767, C227, $D$2:$D$767, D227, $E$2:$E$767, E227) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11554,7 +11532,7 @@
       </c>
       <c r="J228" s="40"/>
       <c r="N228" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B228, $C$2:$C$767, C228, $D$2:$D$767, D228, $E$2:$E$767, E228) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11588,7 +11566,7 @@
       </c>
       <c r="J229" s="40"/>
       <c r="N229" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B229, $C$2:$C$767, C229, $D$2:$D$767, D229, $E$2:$E$767, E229) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O229" s="35"/>
@@ -11625,7 +11603,7 @@
         <v>118</v>
       </c>
       <c r="N230" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B230, $C$2:$C$767, C230, $D$2:$D$767, D230, $E$2:$E$767, E230) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11659,7 +11637,7 @@
       </c>
       <c r="J231" s="40"/>
       <c r="N231" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B231, $C$2:$C$767, C231, $D$2:$D$767, D231, $E$2:$E$767, E231) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11705,7 +11683,7 @@
         <v>260</v>
       </c>
       <c r="N232" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B232, $C$2:$C$767, C232, $D$2:$D$767, D232, $E$2:$E$767, E232) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11739,7 +11717,7 @@
       </c>
       <c r="J233" s="40"/>
       <c r="N233" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B233, $C$2:$C$767, C233, $D$2:$D$767, D233, $E$2:$E$767, E233) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11785,7 +11763,7 @@
         <v>250</v>
       </c>
       <c r="N234" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B234, $C$2:$C$767, C234, $D$2:$D$767, D234, $E$2:$E$767, E234) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11831,7 +11809,7 @@
         <v>300</v>
       </c>
       <c r="N235" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B235, $C$2:$C$767, C235, $D$2:$D$767, D235, $E$2:$E$767, E235) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11867,7 +11845,7 @@
         <v>117</v>
       </c>
       <c r="N236" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B236, $C$2:$C$767, C236, $D$2:$D$767, D236, $E$2:$E$767, E236) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11901,7 +11879,7 @@
       </c>
       <c r="J237" s="40"/>
       <c r="N237" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B237, $C$2:$C$767, C237, $D$2:$D$767, D237, $E$2:$E$767, E237) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11947,7 +11925,7 @@
         <v>300</v>
       </c>
       <c r="N238" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B238, $C$2:$C$767, C238, $D$2:$D$767, D238, $E$2:$E$767, E238) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11983,7 +11961,7 @@
         <v>55</v>
       </c>
       <c r="N239" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B239, $C$2:$C$767, C239, $D$2:$D$767, D239, $E$2:$E$767, E239) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12019,7 +11997,7 @@
         <v>117</v>
       </c>
       <c r="N240" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B240, $C$2:$C$767, C240, $D$2:$D$767, D240, $E$2:$E$767, E240) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P240" s="35"/>
@@ -12066,7 +12044,7 @@
         <v>650</v>
       </c>
       <c r="N241" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B241, $C$2:$C$767, C241, $D$2:$D$767, D241, $E$2:$E$767, E241) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P241" s="35"/>
@@ -12103,7 +12081,7 @@
         <v>118</v>
       </c>
       <c r="N242" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B242, $C$2:$C$767, C242, $D$2:$D$767, D242, $E$2:$E$767, E242) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12139,7 +12117,7 @@
         <v>118</v>
       </c>
       <c r="N243" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B243, $C$2:$C$767, C243, $D$2:$D$767, D243, $E$2:$E$767, E243) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O243" s="35"/>
@@ -12176,7 +12154,7 @@
         <v>118</v>
       </c>
       <c r="N244" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B244, $C$2:$C$767, C244, $D$2:$D$767, D244, $E$2:$E$767, E244) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12213,7 +12191,7 @@
       <c r="L245" s="18"/>
       <c r="M245" s="18"/>
       <c r="N245" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B245, $C$2:$C$767, C245, $D$2:$D$767, D245, $E$2:$E$767, E245) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O245" s="10"/>
@@ -12251,7 +12229,7 @@
         <v>117</v>
       </c>
       <c r="N246" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B246, $C$2:$C$767, C246, $D$2:$D$767, D246, $E$2:$E$767, E246) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12297,7 +12275,7 @@
         <v>285</v>
       </c>
       <c r="N247" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B247, $C$2:$C$767, C247, $D$2:$D$767, D247, $E$2:$E$767, E247) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12343,7 +12321,7 @@
         <v>726</v>
       </c>
       <c r="N248" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B248, $C$2:$C$767, C248, $D$2:$D$767, D248, $E$2:$E$767, E248) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12382,7 +12360,7 @@
         <v>146</v>
       </c>
       <c r="N249" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B249, $C$2:$C$767, C249, $D$2:$D$767, D249, $E$2:$E$767, E249) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12416,7 +12394,7 @@
       </c>
       <c r="J250" s="40"/>
       <c r="N250" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B250, $C$2:$C$767, C250, $D$2:$D$767, D250, $E$2:$E$767, E250) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12450,7 +12428,7 @@
       </c>
       <c r="J251" s="40"/>
       <c r="N251" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B251, $C$2:$C$767, C251, $D$2:$D$767, D251, $E$2:$E$767, E251) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12484,7 +12462,7 @@
       </c>
       <c r="J252" s="40"/>
       <c r="N252" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B252, $C$2:$C$767, C252, $D$2:$D$767, D252, $E$2:$E$767, E252) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12530,7 +12508,7 @@
         <v>300</v>
       </c>
       <c r="N253" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B253, $C$2:$C$767, C253, $D$2:$D$767, D253, $E$2:$E$767, E253) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12576,7 +12554,7 @@
         <v>300</v>
       </c>
       <c r="N254" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B254, $C$2:$C$767, C254, $D$2:$D$767, D254, $E$2:$E$767, E254) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O254" s="10"/>
@@ -12612,7 +12590,7 @@
       </c>
       <c r="J255" s="40"/>
       <c r="N255" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B255, $C$2:$C$767, C255, $D$2:$D$767, D255, $E$2:$E$767, E255) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12658,7 +12636,7 @@
         <v>275</v>
       </c>
       <c r="N256" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B256, $C$2:$C$767, C256, $D$2:$D$767, D256, $E$2:$E$767, E256) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12692,7 +12670,7 @@
       </c>
       <c r="J257" s="40"/>
       <c r="N257" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B257, $C$2:$C$767, C257, $D$2:$D$767, D257, $E$2:$E$767, E257) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12728,7 +12706,7 @@
         <v>118</v>
       </c>
       <c r="N258" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B258, $C$2:$C$767, C258, $D$2:$D$767, D258, $E$2:$E$767, E258) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N258:N291" si="10">IF(COUNTIFS( $B$2:$B$767, B258, $C$2:$C$767, C258, $D$2:$D$767, D258, $E$2:$E$767, E258) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -12762,7 +12740,7 @@
       </c>
       <c r="J259" s="40"/>
       <c r="N259" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B259, $C$2:$C$767, C259, $D$2:$D$767, D259, $E$2:$E$767, E259) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12798,7 +12776,7 @@
         <v>118</v>
       </c>
       <c r="N260" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B260, $C$2:$C$767, C260, $D$2:$D$767, D260, $E$2:$E$767, E260) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
       <c r="O260" s="35"/>
@@ -12835,7 +12813,7 @@
         <v>118</v>
       </c>
       <c r="N261" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B261, $C$2:$C$767, C261, $D$2:$D$767, D261, $E$2:$E$767, E261) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12881,7 +12859,7 @@
         <v>480</v>
       </c>
       <c r="N262" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B262, $C$2:$C$767, C262, $D$2:$D$767, D262, $E$2:$E$767, E262) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12915,7 +12893,7 @@
       </c>
       <c r="J263" s="40"/>
       <c r="N263" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B263, $C$2:$C$767, C263, $D$2:$D$767, D263, $E$2:$E$767, E263) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
       <c r="P263" s="35"/>
@@ -12950,7 +12928,7 @@
       </c>
       <c r="J264" s="40"/>
       <c r="N264" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B264, $C$2:$C$767, C264, $D$2:$D$767, D264, $E$2:$E$767, E264) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12986,7 +12964,7 @@
         <v>118</v>
       </c>
       <c r="N265" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B265, $C$2:$C$767, C265, $D$2:$D$767, D265, $E$2:$E$767, E265) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13032,7 +13010,7 @@
         <v>250</v>
       </c>
       <c r="N266" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B266, $C$2:$C$767, C266, $D$2:$D$767, D266, $E$2:$E$767, E266) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
       <c r="P266" s="35"/>
@@ -13069,7 +13047,7 @@
         <v>117</v>
       </c>
       <c r="N267" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B267, $C$2:$C$767, C267, $D$2:$D$767, D267, $E$2:$E$767, E267) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13105,7 +13083,7 @@
         <v>118</v>
       </c>
       <c r="N268" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B268, $C$2:$C$767, C268, $D$2:$D$767, D268, $E$2:$E$767, E268) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13139,7 +13117,7 @@
       </c>
       <c r="J269" s="40"/>
       <c r="N269" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B269, $C$2:$C$767, C269, $D$2:$D$767, D269, $E$2:$E$767, E269) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13185,7 +13163,7 @@
         <v>300</v>
       </c>
       <c r="N270" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B270, $C$2:$C$767, C270, $D$2:$D$767, D270, $E$2:$E$767, E270) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13219,7 +13197,7 @@
       </c>
       <c r="J271" s="40"/>
       <c r="N271" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B271, $C$2:$C$767, C271, $D$2:$D$767, D271, $E$2:$E$767, E271) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13253,7 +13231,7 @@
       </c>
       <c r="J272" s="40"/>
       <c r="N272" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B272, $C$2:$C$767, C272, $D$2:$D$767, D272, $E$2:$E$767, E272) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13287,7 +13265,7 @@
       </c>
       <c r="J273" s="40"/>
       <c r="N273" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B273, $C$2:$C$767, C273, $D$2:$D$767, D273, $E$2:$E$767, E273) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
       <c r="O273" s="35"/>
@@ -13322,7 +13300,7 @@
       </c>
       <c r="J274" s="40"/>
       <c r="N274" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B274, $C$2:$C$767, C274, $D$2:$D$767, D274, $E$2:$E$767, E274) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13358,7 +13336,7 @@
         <v>118</v>
       </c>
       <c r="N275" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B275, $C$2:$C$767, C275, $D$2:$D$767, D275, $E$2:$E$767, E275) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13392,7 +13370,7 @@
       </c>
       <c r="J276" s="40"/>
       <c r="N276" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B276, $C$2:$C$767, C276, $D$2:$D$767, D276, $E$2:$E$767, E276) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13438,7 +13416,7 @@
         <v>250</v>
       </c>
       <c r="N277" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B277, $C$2:$C$767, C277, $D$2:$D$767, D277, $E$2:$E$767, E277) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13472,7 +13450,7 @@
       </c>
       <c r="J278" s="40"/>
       <c r="N278" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B278, $C$2:$C$767, C278, $D$2:$D$767, D278, $E$2:$E$767, E278) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13506,7 +13484,7 @@
       </c>
       <c r="J279" s="40"/>
       <c r="N279" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B279, $C$2:$C$767, C279, $D$2:$D$767, D279, $E$2:$E$767, E279) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
       <c r="P279" s="35"/>
@@ -13541,7 +13519,7 @@
       </c>
       <c r="J280" s="40"/>
       <c r="N280" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B280, $C$2:$C$767, C280, $D$2:$D$767, D280, $E$2:$E$767, E280) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13575,7 +13553,7 @@
       </c>
       <c r="J281" s="40"/>
       <c r="N281" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B281, $C$2:$C$767, C281, $D$2:$D$767, D281, $E$2:$E$767, E281) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13609,7 +13587,7 @@
       </c>
       <c r="J282" s="40"/>
       <c r="N282" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B282, $C$2:$C$767, C282, $D$2:$D$767, D282, $E$2:$E$767, E282) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13645,7 +13623,7 @@
         <v>118</v>
       </c>
       <c r="N283" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B283, $C$2:$C$767, C283, $D$2:$D$767, D283, $E$2:$E$767, E283) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13681,7 +13659,7 @@
         <v>55</v>
       </c>
       <c r="N284" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B284, $C$2:$C$767, C284, $D$2:$D$767, D284, $E$2:$E$767, E284) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13717,7 +13695,7 @@
         <v>118</v>
       </c>
       <c r="N285" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B285, $C$2:$C$767, C285, $D$2:$D$767, D285, $E$2:$E$767, E285) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13751,7 +13729,7 @@
       </c>
       <c r="J286" s="40"/>
       <c r="N286" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B286, $C$2:$C$767, C286, $D$2:$D$767, D286, $E$2:$E$767, E286) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13797,7 +13775,7 @@
         <v>250</v>
       </c>
       <c r="N287" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B287, $C$2:$C$767, C287, $D$2:$D$767, D287, $E$2:$E$767, E287) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13831,7 +13809,7 @@
       </c>
       <c r="J288" s="40"/>
       <c r="N288" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B288, $C$2:$C$767, C288, $D$2:$D$767, D288, $E$2:$E$767, E288) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13865,7 +13843,7 @@
       </c>
       <c r="J289" s="40"/>
       <c r="N289" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B289, $C$2:$C$767, C289, $D$2:$D$767, D289, $E$2:$E$767, E289) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13899,7 +13877,7 @@
       </c>
       <c r="J290" s="40"/>
       <c r="N290" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B290, $C$2:$C$767, C290, $D$2:$D$767, D290, $E$2:$E$767, E290) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
       <c r="O290" s="35"/>
@@ -13934,7 +13912,7 @@
       </c>
       <c r="J291" s="40"/>
       <c r="N291" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$767, B291, $C$2:$C$767, C291, $D$2:$D$767, D291, $E$2:$E$767, E291) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="10"/>
         <v>Unique</v>
       </c>
     </row>

</xml_diff>